<commit_message>
Added two more hypothesis testing with the mean population exercises.
</commit_message>
<xml_diff>
--- a/resources/Part_3_Statistics/S20_L130/4.7.Test-for-the-mean.Dependent-samples-exercise.xlsx
+++ b/resources/Part_3_Statistics/S20_L130/4.7.Test-for-the-mean.Dependent-samples-exercise.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="18229"/>
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Weight-loss data, lbs" sheetId="1" r:id="rId1"/>
     <sheet name="Weight-loss data, kg" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="162913"/>
   <fileRecoveryPr autoRecover="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="31">
   <si>
     <t>Test the mean. Dependent Samples</t>
   </si>
@@ -78,6 +78,84 @@
   </si>
   <si>
     <t>After (kg)</t>
+  </si>
+  <si>
+    <t>Difference(kg)(Task1)</t>
+  </si>
+  <si>
+    <t>: 0&gt;=before -after</t>
+  </si>
+  <si>
+    <r>
+      <t>We want to prove that the program works, so H</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> shall be that it does not work, that "after"&gt;="before"</t>
+    </r>
+  </si>
+  <si>
+    <t>Small sample, Std Dev unknown, assumed equal. Use the T-Statistic</t>
+  </si>
+  <si>
+    <r>
+      <t>This is a one-sided test, since all values greater than 0 discard H</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Diff. Mean</t>
+  </si>
+  <si>
+    <t>Diff. Std Dev</t>
+  </si>
+  <si>
+    <t>Std err</t>
+  </si>
+  <si>
+    <t>T-Score</t>
+  </si>
+  <si>
+    <t>p-value</t>
+  </si>
+  <si>
+    <t>We can reject the H0 hypothesis with a 5% significance level, but not with a 1% significance level.</t>
+  </si>
+  <si>
+    <t>we can reject the H0 hypothesis with a 3,8% significance level.</t>
   </si>
 </sst>
 </file>
@@ -87,7 +165,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -112,6 +190,13 @@
       <b/>
       <sz val="9"/>
       <color rgb="FF002060"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <vertAlign val="subscript"/>
+      <sz val="9"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -458,36 +543,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:N25"/>
-  <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.21875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.88671875" style="1"/>
-    <col min="6" max="6" width="15.77734375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="14" width="8.88671875" style="1"/>
-    <col min="15" max="15" width="2.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="10.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.85546875" style="1"/>
+    <col min="6" max="6" width="15.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="14" width="8.85546875" style="1"/>
+    <col min="15" max="15" width="2.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="2:14" ht="12" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="2:14" ht="12" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B3" s="3"/>
     </row>
-    <row r="4" spans="2:14" ht="12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
@@ -495,7 +580,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:14" ht="12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
@@ -503,7 +588,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:14" ht="12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B6" s="3" t="s">
         <v>4</v>
       </c>
@@ -511,7 +596,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="2:14" ht="12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B7" s="3" t="s">
         <v>6</v>
       </c>
@@ -519,7 +604,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="2:14" ht="12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
@@ -527,7 +612,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="2:14" ht="12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B9" s="3" t="s">
         <v>12</v>
       </c>
@@ -535,7 +620,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="2:14" ht="12.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:14" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
         <v>15</v>
       </c>
@@ -544,7 +629,7 @@
       </c>
       <c r="D11" s="11"/>
     </row>
-    <row r="12" spans="2:14" ht="12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B12" s="5">
         <v>228.5752732416</v>
       </c>
@@ -562,7 +647,7 @@
       <c r="M12" s="8"/>
       <c r="N12" s="8"/>
     </row>
-    <row r="13" spans="2:14" ht="12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B13" s="5">
         <v>244.00763158160001</v>
       </c>
@@ -580,7 +665,7 @@
       <c r="M13" s="8"/>
       <c r="N13" s="8"/>
     </row>
-    <row r="14" spans="2:14" ht="12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B14" s="5">
         <v>262.46032291099999</v>
       </c>
@@ -616,7 +701,7 @@
       <c r="M15" s="8"/>
       <c r="N15" s="8"/>
     </row>
-    <row r="16" spans="2:14" ht="12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B16" s="5">
         <v>202.14184802779999</v>
       </c>
@@ -652,7 +737,7 @@
       <c r="M17" s="8"/>
       <c r="N17" s="8"/>
     </row>
-    <row r="18" spans="2:14" ht="12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B18" s="5">
         <v>195.85867356079999</v>
       </c>
@@ -688,7 +773,7 @@
       <c r="M19" s="8"/>
       <c r="N19" s="8"/>
     </row>
-    <row r="20" spans="2:14" ht="12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B20" s="5">
         <v>243.32419856939998</v>
       </c>
@@ -777,36 +862,36 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:T25"/>
-  <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18.109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="8.88671875" style="1"/>
-    <col min="6" max="6" width="15.77734375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.21875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="7.6640625" style="1" customWidth="1"/>
-    <col min="10" max="14" width="8.88671875" style="1"/>
-    <col min="15" max="15" width="2.6640625" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="10.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.85546875" style="1"/>
+    <col min="6" max="6" width="15.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="7.7109375" style="1" customWidth="1"/>
+    <col min="10" max="14" width="8.85546875" style="1"/>
+    <col min="15" max="15" width="2.7109375" style="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:20" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B2" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B3" s="3"/>
     </row>
-    <row r="4" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
@@ -814,7 +899,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
@@ -822,7 +907,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B6" s="3" t="s">
         <v>4</v>
       </c>
@@ -830,7 +915,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B7" s="3" t="s">
         <v>6</v>
       </c>
@@ -838,7 +923,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
@@ -846,7 +931,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B9" s="3" t="s">
         <v>12</v>
       </c>
@@ -858,41 +943,69 @@
       <c r="S10" s="8"/>
       <c r="T10" s="8"/>
     </row>
-    <row r="11" spans="2:20" ht="12.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:20" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="4" t="s">
         <v>17</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="11"/>
+      <c r="D11" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
+      <c r="F11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="5">
+        <f>AVERAGE(D12:D21)</f>
+        <v>1.1371963718659388</v>
+      </c>
+      <c r="H11" s="3" t="str">
+        <f>B6</f>
+        <v>Task 2</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>21</v>
+      </c>
       <c r="J11" s="8"/>
       <c r="K11" s="8"/>
       <c r="L11" s="8"/>
       <c r="M11" s="8"/>
       <c r="N11" s="8"/>
       <c r="O11" s="8"/>
+      <c r="P11" s="1" t="s">
+        <v>20</v>
+      </c>
       <c r="S11" s="8"/>
       <c r="T11" s="8"/>
     </row>
-    <row r="12" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B12" s="5">
         <v>103.67999991305493</v>
       </c>
       <c r="C12" s="5">
         <v>103.66853616350001</v>
       </c>
-      <c r="D12" s="7"/>
+      <c r="D12" s="7">
+        <f>B12-C12</f>
+        <v>1.1463749554920355E-2</v>
+      </c>
       <c r="E12" s="8"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
+      <c r="F12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="1">
+        <f>_xlfn.STDEV.S(D12:D21)</f>
+        <v>1.7928657175882481</v>
+      </c>
+      <c r="H12" s="3" t="str">
+        <f>B7</f>
+        <v>Task 3</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>22</v>
+      </c>
       <c r="J12" s="8"/>
       <c r="K12" s="8"/>
       <c r="L12" s="8"/>
@@ -902,19 +1015,32 @@
       <c r="S12" s="7"/>
       <c r="T12" s="8"/>
     </row>
-    <row r="13" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:20" ht="13.5" x14ac:dyDescent="0.25">
       <c r="B13" s="5">
         <v>110.67999990718481</v>
       </c>
       <c r="C13" s="5">
         <v>108.38388546481596</v>
       </c>
-      <c r="D13" s="7"/>
+      <c r="D13" s="7">
+        <f t="shared" ref="D13:D21" si="0">B13-C13</f>
+        <v>2.2961144423688467</v>
+      </c>
       <c r="E13" s="8"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="7"/>
+      <c r="F13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" s="1">
+        <f>G12/SQRT(COUNT(D12:D21))</f>
+        <v>0.56695392064110672</v>
+      </c>
+      <c r="H13" s="3" t="str">
+        <f>B8</f>
+        <v>Task 4</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="J13" s="7"/>
       <c r="K13" s="8"/>
       <c r="L13" s="8"/>
@@ -924,19 +1050,32 @@
       <c r="S13" s="7"/>
       <c r="T13" s="8"/>
     </row>
-    <row r="14" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B14" s="5">
         <v>119.04999990016579</v>
       </c>
       <c r="C14" s="5">
         <v>115.9472816194</v>
       </c>
-      <c r="D14" s="7"/>
+      <c r="D14" s="7">
+        <f t="shared" si="0"/>
+        <v>3.1027182807657852</v>
+      </c>
       <c r="E14" s="8"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="7"/>
+      <c r="F14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" s="1">
+        <f>G11/G13</f>
+        <v>2.0058003489595886</v>
+      </c>
+      <c r="H14" s="3" t="str">
+        <f>B9</f>
+        <v>Task 5</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>29</v>
+      </c>
       <c r="J14" s="7"/>
       <c r="K14" s="8"/>
       <c r="L14" s="8"/>
@@ -953,12 +1092,21 @@
       <c r="C15" s="5">
         <v>101.7044812014</v>
       </c>
-      <c r="D15" s="7"/>
+      <c r="D15" s="7">
+        <f t="shared" si="0"/>
+        <v>4.5518713273409617E-2</v>
+      </c>
       <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
+      <c r="F15" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G15" s="8">
+        <v>3.7920000000000002E-2</v>
+      </c>
       <c r="H15" s="8"/>
-      <c r="I15" s="7"/>
+      <c r="I15" s="7" t="s">
+        <v>30</v>
+      </c>
       <c r="J15" s="7"/>
       <c r="K15" s="8"/>
       <c r="L15" s="8"/>
@@ -968,14 +1116,17 @@
       <c r="S15" s="7"/>
       <c r="T15" s="8"/>
     </row>
-    <row r="16" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B16" s="5">
         <v>91.689999923109625</v>
       </c>
       <c r="C16" s="5">
         <v>90.586932212700006</v>
       </c>
-      <c r="D16" s="7"/>
+      <c r="D16" s="7">
+        <f t="shared" si="0"/>
+        <v>1.1030677104096185</v>
+      </c>
       <c r="E16" s="8"/>
       <c r="F16" s="9"/>
       <c r="G16" s="9"/>
@@ -997,7 +1148,10 @@
       <c r="C17" s="5">
         <v>112.70388546119325</v>
       </c>
-      <c r="D17" s="7"/>
+      <c r="D17" s="7">
+        <f t="shared" si="0"/>
+        <v>-0.67388555514055781</v>
+      </c>
       <c r="E17" s="8"/>
       <c r="F17" s="8"/>
       <c r="G17" s="8"/>
@@ -1012,14 +1166,17 @@
       <c r="S17" s="7"/>
       <c r="T17" s="8"/>
     </row>
-    <row r="18" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B18" s="5">
         <v>88.839999925499612</v>
       </c>
       <c r="C18" s="5">
         <v>87.363885482443138</v>
       </c>
-      <c r="D18" s="7"/>
+      <c r="D18" s="7">
+        <f t="shared" si="0"/>
+        <v>1.4761144430564741</v>
+      </c>
       <c r="E18" s="8"/>
       <c r="F18" s="9"/>
       <c r="G18" s="9"/>
@@ -1041,7 +1198,10 @@
       <c r="C19" s="5">
         <v>103.8038854686567</v>
       </c>
-      <c r="D19" s="7"/>
+      <c r="D19" s="7">
+        <f t="shared" si="0"/>
+        <v>1.376114443140338</v>
+      </c>
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
       <c r="G19" s="8"/>
@@ -1056,14 +1216,17 @@
       <c r="S19" s="7"/>
       <c r="T19" s="8"/>
     </row>
-    <row r="20" spans="2:20" ht="12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B20" s="5">
         <v>110.36999990744475</v>
       </c>
       <c r="C20" s="5">
         <v>106.07388546675311</v>
       </c>
-      <c r="D20" s="7"/>
+      <c r="D20" s="7">
+        <f t="shared" si="0"/>
+        <v>4.2961144406916389</v>
+      </c>
       <c r="E20" s="8"/>
       <c r="F20" s="9"/>
       <c r="G20" s="11"/>
@@ -1085,7 +1248,10 @@
       <c r="C21" s="6">
         <v>122.651376848</v>
       </c>
-      <c r="D21" s="7"/>
+      <c r="D21" s="6">
+        <f t="shared" si="0"/>
+        <v>-1.6613769494610864</v>
+      </c>
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
       <c r="G21" s="10"/>

</xml_diff>